<commit_message>
Add 'constraints_detailed' 'requisito_clase' plus correction archives
</commit_message>
<xml_diff>
--- a/db/tabla_minable.xlsx
+++ b/db/tabla_minable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PosGrado\Proyecto Titulacion\Timetabling\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PosGrado\Proyecto Titulacion\Timetabling\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100808CB-CEDA-46E8-B6E7-88E2D5AF70A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA8BC4C-099E-4AB6-8D90-71826D66292C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="5040" windowWidth="28785" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="600" yWindow="2790" windowWidth="28785" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>